<commit_message>
ADD: new price from 22.08.2026
</commit_message>
<xml_diff>
--- a/SPLIT_COMPANY_DATA/RESULT/companies_result/КМЕТСТВО ЗВЕЗДИЦА/КМЕТСТВО ЗВЕЗДИЦА.xlsx
+++ b/SPLIT_COMPANY_DATA/RESULT/companies_result/КМЕТСТВО ЗВЕЗДИЦА/КМЕТСТВО ЗВЕЗДИЦА.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
   <si>
     <t>Дата</t>
   </si>
@@ -34,9 +34,6 @@
     <t>Литри</t>
   </si>
   <si>
-    <t>Тип количество</t>
-  </si>
-  <si>
     <t>GTA цена</t>
   </si>
   <si>
@@ -58,37 +55,25 @@
     <t>Billing_Document</t>
   </si>
   <si>
-    <t>1148 Варна пристанище</t>
-  </si>
-  <si>
-    <t>ТубаЗвездица</t>
+    <t>Варна Порт</t>
+  </si>
+  <si>
+    <t>Варна Евkсиноград</t>
   </si>
   <si>
     <t>В0583ВТ</t>
   </si>
   <si>
-    <t>78970155027722747</t>
-  </si>
-  <si>
     <t>78970155027721806</t>
   </si>
   <si>
-    <t>95 EKONOMY UNLEADED</t>
-  </si>
-  <si>
     <t>E GAS LPG</t>
   </si>
   <si>
-    <t>L15</t>
-  </si>
-  <si>
-    <t>08:57:00</t>
-  </si>
-  <si>
-    <t>3235235182 3235235182</t>
-  </si>
-  <si>
-    <t>3235235386 3235235386</t>
+    <t>10:07</t>
+  </si>
+  <si>
+    <t>16:52</t>
   </si>
   <si>
     <t>Общи литри по продукт / КМЕТСТВО ЗВЕЗДИЦА</t>
@@ -114,9 +99,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="#,##0.000"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00000"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -210,10 +195,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -508,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -517,17 +502,16 @@
     <col min="4" max="4" width="28.7109375" customWidth="1"/>
     <col min="5" max="5" width="22.7109375" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="23.7109375" customWidth="1"/>
     <col min="9" max="9" width="15.7109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="23.7109375" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" customWidth="1"/>
-    <col min="14" max="14" width="23.7109375" customWidth="1"/>
+    <col min="11" max="11" width="7.7109375" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:13">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -567,101 +551,92 @@
       <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="3">
+        <v>46239</v>
+      </c>
+      <c r="B2" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2" s="3">
-        <v>46226</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
       </c>
       <c r="C2" t="s">
         <v>15</v>
       </c>
       <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" t="s">
-        <v>19</v>
-      </c>
       <c r="F2">
-        <v>20</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
+        <v>24.818</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0.65</v>
       </c>
       <c r="H2">
-        <v>1.51</v>
+        <v>16.132</v>
       </c>
       <c r="I2" s="1">
-        <v>30.2</v>
+        <v>0.66</v>
       </c>
       <c r="J2">
-        <v>1.54</v>
-      </c>
-      <c r="K2" s="1">
-        <v>30.8</v>
-      </c>
-      <c r="L2" t="s">
-        <v>22</v>
+        <v>16.38</v>
+      </c>
+      <c r="K2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2">
+        <v>120480</v>
       </c>
       <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2" t="s">
-        <v>23</v>
+        <v>242429</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:13">
       <c r="A3" s="3">
-        <v>46226</v>
+        <v>46242</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
       </c>
       <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s">
-        <v>18</v>
-      </c>
       <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3">
+        <v>16.652</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="H3">
+        <v>10.824</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0.66</v>
+      </c>
+      <c r="J3">
+        <v>10.99</v>
+      </c>
+      <c r="K3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3">
+        <v>12064</v>
+      </c>
+      <c r="M3">
+        <v>236290</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="F3">
-        <v>23.406</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3">
-        <v>0.63</v>
-      </c>
-      <c r="I3" s="1">
-        <v>14.746</v>
-      </c>
-      <c r="J3">
-        <v>0.64</v>
-      </c>
-      <c r="K3" s="1">
-        <v>14.98</v>
-      </c>
-      <c r="L3" t="s">
-        <v>22</v>
-      </c>
-      <c r="M3">
-        <v>12018</v>
-      </c>
-      <c r="N3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
-      <c r="A6" s="4" t="s">
-        <v>25</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -669,82 +644,62 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:13">
       <c r="A7" s="5" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:13">
       <c r="A8" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B8" s="7">
-        <v>23.406</v>
-      </c>
-      <c r="C8" s="8">
-        <v>1</v>
+        <v>41.47</v>
+      </c>
+      <c r="C8" s="7">
+        <v>2</v>
       </c>
       <c r="D8" s="8">
-        <v>0.63</v>
-      </c>
-      <c r="E8" s="8">
-        <v>14.746</v>
-      </c>
-      <c r="F8" s="8">
-        <v>14.98</v>
+        <v>0.65001</v>
+      </c>
+      <c r="E8" s="7">
+        <v>26.96</v>
+      </c>
+      <c r="F8" s="7">
+        <v>27.37</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
-      <c r="A9" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="7">
-        <v>20</v>
-      </c>
-      <c r="C9" s="8">
-        <v>1</v>
-      </c>
-      <c r="D9" s="8">
-        <v>1.51</v>
-      </c>
-      <c r="E9" s="8">
-        <v>30.2</v>
-      </c>
-      <c r="F9" s="8">
-        <v>30.8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" s="10">
-        <v>43.406</v>
-      </c>
-      <c r="C10" s="10">
+    <row r="9" spans="1:13">
+      <c r="A9" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="10">
+        <v>41.47</v>
+      </c>
+      <c r="C9" s="10">
         <v>2</v>
       </c>
-      <c r="D10" s="8"/>
-      <c r="E10" s="10">
-        <v>44.946</v>
-      </c>
-      <c r="F10" s="10">
-        <v>45.78</v>
+      <c r="D9" s="8"/>
+      <c r="E9" s="10">
+        <v>26.96</v>
+      </c>
+      <c r="F9" s="10">
+        <v>27.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>